<commit_message>
fix bug in case 2 not being added to matches
</commit_message>
<xml_diff>
--- a/splists_out/needs_revision/BCI_SPECIES_POSSIBLY_WOODY_2026-03-26.xlsx
+++ b/splists_out/needs_revision/BCI_SPECIES_POSSIBLY_WOODY_2026-03-26.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -773,81 +773,81 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cestrum megalophyllum</t>
+          <t>Chamissoa altissima</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cestrum megalophyllum</t>
+          <t>Chamissoa altissima</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Cestrum megalophyllum</t>
+          <t>Chamissoa altissima</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Solanaceae</t>
+          <t>Amaranthaceae</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>shrub or tree</t>
+          <t>scrambling subshrub or shrub</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Chamissoa altissima</t>
+          <t>Clibadium surinamense</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Chamissoa altissima</t>
+          <t>Clibadium surinamense</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Chamissoa altissima</t>
+          <t>Clibadium surinamense</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Amaranthaceae</t>
+          <t>Asteraceae</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>scrambling subshrub or shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>Sw</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Clibadium surinamense</t>
+          <t>Clibadium sylvestre</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Clibadium surinamense</t>
+          <t>Clibadium sylvestre</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Clibadium surinamense</t>
+          <t>Clibadium sylvestre</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>scrambling shrub or tree</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -869,59 +869,59 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Clibadium sylvestre</t>
+          <t>Corchorus siliquosus</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Clibadium sylvestre</t>
+          <t>Corchorus siliquosus</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Clibadium sylvestre</t>
+          <t>Corchorus siliquosus</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>scrambling shrub or tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Sw</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Clusia pratensis</t>
+          <t>Coussapoa asperifolia subsp. magnifolia</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Clusia pratensis</t>
+          <t>Coussapoa asperifolia subsp. magnifolia</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Clusia pratensis</t>
+          <t>Coussapoa asperifolia subsp. magnifolia</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Clusiaceae</t>
+          <t>Urticaceae</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>shrub or tree</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -933,22 +933,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Corchorus siliquosus</t>
+          <t>Crotalaria cajanifolia</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Corchorus siliquosus</t>
+          <t>Crotalaria cajanifolia</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Corchorus siliquosus</t>
+          <t>Crotalaria cajanifolia</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -965,81 +965,81 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Coussapoa asperifolia subsp. magnifolia</t>
+          <t>Dalbergia brownei</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Coussapoa asperifolia subsp. magnifolia</t>
+          <t>Dalbergia brownei</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Coussapoa asperifolia subsp. magnifolia</t>
+          <t>Dalbergia brownei</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Urticaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>shrub or tree</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>L</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Crotalaria cajanifolia</t>
+          <t>Dendropanax stenodontus</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Crotalaria cajanifolia</t>
+          <t>Dendropanax stenodontus</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Crotalaria cajanifolia</t>
+          <t>Dendropanax stenodontus</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Araliaceae</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>shrub or tree</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>S</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Dalbergia brownei</t>
+          <t>Desmodium cajanifolium</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dalbergia brownei</t>
+          <t>Desmodium cajanifolium</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Dalbergia brownei</t>
+          <t>Desmodium cajanifolium</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1049,61 +1049,61 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>shrub or tree</t>
+          <t>perennial or shrub</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>Sw</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Dendropanax stenodontus</t>
+          <t>Desmodium distortum</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Dendropanax stenodontus</t>
+          <t>Desmodium distortum</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Dendropanax stenodontus</t>
+          <t>Desmodium distortum</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Araliaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>shrub or tree</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Desmodium cajanifolium</t>
+          <t>Desmodium wydlerianum</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Desmodium cajanifolium</t>
+          <t>Desmodium wydlerianum</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Desmodium cajanifolium</t>
+          <t>Desmodium wydlerianum</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1113,34 +1113,34 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>perennial or shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Sw</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Desmodium distortum</t>
+          <t>Dieffenbachia longispatha</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Desmodium distortum</t>
+          <t>Dieffenbachia longispatha</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Desmodium distortum</t>
+          <t>Dieffenbachia longispatha</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Araceae</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1150,290 +1150,290 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Desmodium wydlerianum</t>
+          <t>Ficus dugandii</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Desmodium wydlerianum</t>
+          <t>Ficus dugandii</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Desmodium wydlerianum</t>
+          <t>Ficus dugandii</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Moraceae</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>TE</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Dieffenbachia longispatha</t>
+          <t>Hebeclinium macrophyllum</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Dieffenbachia longispatha</t>
+          <t>Hebeclinium macrophyllum</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Dieffenbachia longispatha</t>
+          <t>Hebeclinium macrophyllum</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Araceae</t>
+          <t>Asteraceae</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ficus bullenei</t>
+          <t>Herpetacanthus panamensis</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Ficus bullenei</t>
+          <t>Herpetacanthus panamensis</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Ficus bullenei</t>
+          <t>Herpetacanthus panamensis</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Moraceae</t>
+          <t>Acanthaceae</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Ficus dugandii</t>
+          <t>Hibiscus sororius</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Ficus dugandii</t>
+          <t>Hibiscus sororius</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Ficus dugandii</t>
+          <t>Hibiscus sororius</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Moraceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>Ha</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Hebeclinium macrophyllum</t>
+          <t>Hoffmannia nicotianifolia</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Hebeclinium macrophyllum</t>
+          <t>Hoffmannia nicotianifolia</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Hebeclinium macrophyllum</t>
+          <t>Hoffmannia nicotianifolia</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Rubiaceae</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Herpetacanthus panamensis</t>
+          <t>Indigofera trita subsp. scabra</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Herpetacanthus panamensis</t>
+          <t>Indigofera trita subsp. scabra</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Herpetacanthus panamensis</t>
+          <t>Indigofera subulata var. scabra</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Acanthaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>scrambling subshrub or shrub</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Hibiscus sororius</t>
+          <t>Iresine angustifolia</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Hibiscus sororius</t>
+          <t>Iresine angustifolia</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Hibiscus sororius</t>
+          <t>Iresine angustifolia</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Amaranthaceae</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Ha</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Hoffmannia nicotianifolia</t>
+          <t>Iresine diffusa var. diffusa</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Hoffmannia nicotianifolia</t>
+          <t>Iresine diffusa f. diffusa</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Hoffmannia nicotianifolia</t>
+          <t>Iresine diffusa f. diffusa</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Rubiaceae</t>
+          <t>Amaranthaceae</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Indigofera trita subsp. scabra</t>
+          <t>Kohleria tubiflora</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Indigofera trita subsp. scabra</t>
+          <t>Kohleria tubiflora</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Indigofera subulata var. scabra</t>
+          <t>Kohleria tubiflora</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Gesneriaceae</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>scrambling subshrub or shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1445,182 +1445,182 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Iresine angustifolia</t>
+          <t>Lepidaploa canescens</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Iresine angustifolia</t>
+          <t>Lepidaploa canescens</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Iresine angustifolia</t>
+          <t>Lepidaploa canescens</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Amaranthaceae</t>
+          <t>Asteraceae</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>scrambling shrub or liana</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>Sw</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Iresine diffusa var. diffusa</t>
+          <t>Machaerium darienense</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Iresine diffusa f. diffusa</t>
+          <t>Machaerium darienense</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Iresine diffusa f. diffusa</t>
+          <t>Machaerium darienense</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Amaranthaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>L</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Kohleria tubiflora</t>
+          <t>Manettia reclinata</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Kohleria tubiflora</t>
+          <t>Manettia reclinata</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Kohleria tubiflora</t>
+          <t>Manettia reclinata</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Gesneriaceae</t>
+          <t>Rubiaceae</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>climbing shrub</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>Vw</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Lepidaploa canescens</t>
+          <t>Melochia lupulina</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Lepidaploa canescens</t>
+          <t>Melochia lupulina</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Lepidaploa canescens</t>
+          <t>Melochia lupulina</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>scrambling shrub or liana</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Sw</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Machaerium darienense</t>
+          <t>Melochia melissifolia</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Machaerium darienense</t>
+          <t>Melochia melissifolia</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Machaerium darienense</t>
+          <t>Melochia melissifolia</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Manettia reclinata</t>
+          <t>Mimosa casta</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Manettia reclinata</t>
+          <t>Mimosa casta</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Manettia reclinata</t>
+          <t>Mimosa casta</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Rubiaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1637,214 +1637,214 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Melochia lupulina</t>
+          <t>Mimosa pigra</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Melochia lupulina</t>
+          <t>Mimosa pigra</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Melochia lupulina</t>
+          <t>Mimosa pigra</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>S</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Melochia melissifolia</t>
+          <t>Montrichardia arborescens</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Melochia melissifolia</t>
+          <t>Montrichardia arborescens</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Melochia melissifolia</t>
+          <t>Montrichardia arborescens</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Araceae</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>shrub or tree</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>Sa</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Miconia serrulata</t>
+          <t>Notopleura uliginosa</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Miconia serrulata</t>
+          <t>Notopleura uliginosa</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Miconia serrulata</t>
+          <t>Notopleura uliginosa</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Melastomataceae</t>
+          <t>Rubiaceae</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Mimosa casta</t>
+          <t>Pavonia castaneifolia</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Mimosa casta</t>
+          <t>Pavonia castaneifolia</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Mimosa casta</t>
+          <t>Pavonia castaneifolia</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>climbing shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Vw</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Mimosa pigra</t>
+          <t>Pavonia paniculata</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Mimosa pigra</t>
+          <t>Pavonia paniculata</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Mimosa pigra</t>
+          <t>Pavonia paniculata</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Montrichardia arborescens</t>
+          <t>Pavonia schiedeana</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Montrichardia arborescens</t>
+          <t>Pavonia schiedeana</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Montrichardia arborescens</t>
+          <t>Pavonia schiedeana</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Araceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>shrub or tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Sa</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Notopleura uliginosa</t>
+          <t>Petiveria alliacea</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Notopleura uliginosa</t>
+          <t>Petiveria alliacea</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Notopleura uliginosa</t>
+          <t>Petiveria alliacea</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Rubiaceae</t>
+          <t>Petiveriaceae</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -1861,59 +1861,59 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Pavonia castaneifolia</t>
+          <t>Phoradendron quadrangulare</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Pavonia castaneifolia</t>
+          <t>Phoradendron quadrangulare</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Pavonia castaneifolia</t>
+          <t>Phoradendron quadrangulare</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Santalaceae</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>hemiparasitic shrub</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>PE</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Pavonia paniculata</t>
+          <t>Phytolacca rivinoides</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Pavonia paniculata</t>
+          <t>Phytolacca rivinoides</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Pavonia paniculata</t>
+          <t>Phytolacca rivinoides</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Phytolaccaceae</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>perennial or shrub</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -1925,22 +1925,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Pavonia schiedeana</t>
+          <t>Piper darienense</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Pavonia schiedeana</t>
+          <t>Piper darienense</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Pavonia schiedeana</t>
+          <t>Piper darienense</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Piperaceae</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -1957,27 +1957,27 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Petiveria alliacea</t>
+          <t>Piper pseudogaragaranum</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Petiveria alliacea</t>
+          <t>Piper pseudogaragaranum</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Petiveria alliacea</t>
+          <t>Piper pseudogaragaranum</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Petiveriaceae</t>
+          <t>Piperaceae</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -1989,81 +1989,81 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Phoradendron quadrangulare</t>
+          <t>Piper pubistipulum</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Phoradendron quadrangulare</t>
+          <t>Piper pubistipulum</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Phoradendron quadrangulare</t>
+          <t>Piper pubistipulum</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Santalaceae</t>
+          <t>Piperaceae</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>hemiparasitic shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Phytolacca rivinoides</t>
+          <t>Piper trigonum</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Phytolacca rivinoides</t>
+          <t>Piper trigonum</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Phytolacca rivinoides</t>
+          <t>Piper trigonum</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Phytolaccaceae</t>
+          <t>Piperaceae</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>perennial or shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Piper darienense</t>
+          <t>Piper viridicaule</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Piper darienense</t>
+          <t>Piper viridicaule</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Piper darienense</t>
+          <t>Piper viridicaule</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2085,59 +2085,59 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Piper pseudogaragaranum</t>
+          <t>Platymiscium pinnatum subsp. polystachyum</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Piper pseudogaragaranum</t>
+          <t>Platymiscium pinnatum subsp. polystachyum</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Piper pseudogaragaranum</t>
+          <t>Platymiscium pinnatum var. pinnatum</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Piperaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>T</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Piper pubistipulum</t>
+          <t>Psychotria guapilensis</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Piper pubistipulum</t>
+          <t>Psychotria guapilensis</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Piper pubistipulum</t>
+          <t>Palicourea tonduzii</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Piperaceae</t>
+          <t>Rubiaceae</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2149,22 +2149,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Piper trigonum</t>
+          <t>Ronabea emetica</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Piper trigonum</t>
+          <t>Ronabea emetica</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Piper trigonum</t>
+          <t>Ronabea emetica</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Piperaceae</t>
+          <t>Rubiaceae</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2181,382 +2181,190 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Piper viridicaule</t>
+          <t>Schistocarpha eupatorioides</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Piper viridicaule</t>
+          <t>Schistocarpha eupatorioides</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Piper viridicaule</t>
+          <t>Schistocarpha eupatorioides</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Piperaceae</t>
+          <t>Asteraceae</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Platymiscium pinnatum subsp. polystachyum</t>
+          <t>Syngonium podophyllum var. podophyllum</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Platymiscium pinnatum subsp. polystachyum</t>
+          <t>Syngonium podophyllum</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Platymiscium pinnatum var. pinnatum</t>
+          <t>Syngonium podophyllum</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Araceae</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>liana</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>E</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Psychotria guapilensis</t>
+          <t>Tachigali versicolor</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Psychotria guapilensis</t>
+          <t>Tachigali versicolor</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Palicourea tonduzii</t>
+          <t>Tachigali versicolor</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Rubiaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>T</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Ronabea emetica</t>
+          <t>Virola multiflora</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Ronabea emetica</t>
+          <t>Virola multiflora</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Ronabea emetica</t>
+          <t>Virola multiflora</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Rubiaceae</t>
+          <t>Myristicaceae</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>T</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Schistocarpha eupatorioides</t>
+          <t>Xanthosoma helleborifolium</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Schistocarpha eupatorioides</t>
+          <t>Xanthosoma helleborifolium</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Schistocarpha eupatorioides</t>
+          <t>Xanthosoma helleborifolium</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Araceae</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>tuberous subshrub</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Stemmadenia grandiflora</t>
+          <t>Xanthosoma mexicanum</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Stemmadenia grandiflora</t>
+          <t>Xanthosoma mexicanum</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Tabernaemontana grandiflora</t>
+          <t>Xanthosoma mexicanum</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Apocynaceae</t>
+          <t>Araceae</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>shrub or tree</t>
+          <t>tuberous subshrub</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Syngonium podophyllum var. podophyllum</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Syngonium podophyllum</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Syngonium podophyllum</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Araceae</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>liana</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Tachigali versicolor</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Tachigali versicolor</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Tachigali versicolor</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Fabaceae</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>tree</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Virola multiflora</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Virola multiflora</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Virola multiflora</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Myristicaceae</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>tree</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Virola nobilis</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Virola nobilis</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Virola nobilis</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Myristicaceae</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>tree</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Xanthosoma helleborifolium</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Xanthosoma helleborifolium</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Xanthosoma helleborifolium</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>Araceae</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>tuberous subshrub</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Xanthosoma mexicanum</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Xanthosoma mexicanum</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Xanthosoma mexicanum</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Araceae</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>tuberous subshrub</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
         <is>
           <t>Hw</t>
         </is>

</xml_diff>

<commit_message>
viewtaxa is not a reliable source for synonyms
</commit_message>
<xml_diff>
--- a/splists_out/needs_revision/BCI_SPECIES_POSSIBLY_WOODY_2026-03-26.xlsx
+++ b/splists_out/needs_revision/BCI_SPECIES_POSSIBLY_WOODY_2026-03-26.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -773,81 +773,81 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Chamissoa altissima</t>
+          <t>Cestrum megalophyllum</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Chamissoa altissima</t>
+          <t>Cestrum megalophyllum</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Chamissoa altissima</t>
+          <t>Cestrum megalophyllum</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Amaranthaceae</t>
+          <t>Solanaceae</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>scrambling subshrub or shrub</t>
+          <t>shrub or tree</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>S</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Clibadium surinamense</t>
+          <t>Chamissoa altissima</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Clibadium surinamense</t>
+          <t>Chamissoa altissima</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Clibadium surinamense</t>
+          <t>Chamissoa altissima</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Amaranthaceae</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>scrambling subshrub or shrub</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Sw</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Clibadium sylvestre</t>
+          <t>Clibadium surinamense</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Clibadium sylvestre</t>
+          <t>Clibadium surinamense</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Clibadium sylvestre</t>
+          <t>Clibadium surinamense</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>scrambling shrub or tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -869,113 +869,113 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Corchorus siliquosus</t>
+          <t>Clibadium sylvestre</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Corchorus siliquosus</t>
+          <t>Clibadium sylvestre</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Corchorus siliquosus</t>
+          <t>Clibadium sylvestre</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Asteraceae</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>scrambling shrub or tree</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>Sw</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Coussapoa asperifolia subsp. magnifolia</t>
+          <t>Corchorus siliquosus</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Coussapoa asperifolia subsp. magnifolia</t>
+          <t>Corchorus siliquosus</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Coussapoa asperifolia subsp. magnifolia</t>
+          <t>Corchorus siliquosus</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Urticaceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Crotalaria cajanifolia</t>
+          <t>Coussapoa asperifolia subsp. magnifolia</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Crotalaria cajanifolia</t>
+          <t>Coussapoa asperifolia subsp. magnifolia</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Crotalaria cajanifolia</t>
+          <t>Coussapoa asperifolia subsp. magnifolia</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Urticaceae</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>E</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Dalbergia brownei</t>
+          <t>Crotalaria cajanifolia</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Dalbergia brownei</t>
+          <t>Crotalaria cajanifolia</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Dalbergia brownei</t>
+          <t>Crotalaria cajanifolia</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -985,34 +985,34 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>shrub or tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Dendropanax stenodontus</t>
+          <t>Dalbergia brownei</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Dendropanax stenodontus</t>
+          <t>Dalbergia brownei</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Dendropanax stenodontus</t>
+          <t>Dalbergia brownei</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Araliaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1022,56 +1022,56 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Desmodium cajanifolium</t>
+          <t>Dendropanax stenodontus</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Desmodium cajanifolium</t>
+          <t>Dendropanax stenodontus</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Desmodium cajanifolium</t>
+          <t>Dendropanax stenodontus</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Araliaceae</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>perennial or shrub</t>
+          <t>shrub or tree</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Sw</t>
+          <t>S</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Desmodium distortum</t>
+          <t>Desmodium cajanifolium</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Desmodium distortum</t>
+          <t>Desmodium cajanifolium</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Desmodium distortum</t>
+          <t>Desmodium cajanifolium</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1081,29 +1081,29 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>perennial or shrub</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>Sw</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Desmodium wydlerianum</t>
+          <t>Desmodium distortum</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Desmodium wydlerianum</t>
+          <t>Desmodium distortum</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Desmodium wydlerianum</t>
+          <t>Desmodium distortum</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1113,39 +1113,39 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Dieffenbachia longispatha</t>
+          <t>Desmodium wydlerianum</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dieffenbachia longispatha</t>
+          <t>Desmodium wydlerianum</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Dieffenbachia longispatha</t>
+          <t>Desmodium wydlerianum</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Araceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1157,155 +1157,155 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Ficus dugandii</t>
+          <t>Dieffenbachia longispatha</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Ficus dugandii</t>
+          <t>Dieffenbachia longispatha</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ficus dugandii</t>
+          <t>Dieffenbachia longispatha</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Moraceae</t>
+          <t>Araceae</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Hebeclinium macrophyllum</t>
+          <t>Ficus bullenei</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Hebeclinium macrophyllum</t>
+          <t>Ficus bullenei</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Hebeclinium macrophyllum</t>
+          <t>Ficus bullenei</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Moraceae</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>TE</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Herpetacanthus panamensis</t>
+          <t>Ficus dugandii</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Herpetacanthus panamensis</t>
+          <t>Ficus dugandii</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Herpetacanthus panamensis</t>
+          <t>Ficus dugandii</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Acanthaceae</t>
+          <t>Moraceae</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>TE</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Hibiscus sororius</t>
+          <t>Hebeclinium macrophyllum</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Hibiscus sororius</t>
+          <t>Hebeclinium macrophyllum</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Hibiscus sororius</t>
+          <t>Hebeclinium macrophyllum</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Asteraceae</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Ha</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Hoffmannia nicotianifolia</t>
+          <t>Herpetacanthus panamensis</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Hoffmannia nicotianifolia</t>
+          <t>Herpetacanthus panamensis</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Hoffmannia nicotianifolia</t>
+          <t>Herpetacanthus panamensis</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Rubiaceae</t>
+          <t>Acanthaceae</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1317,91 +1317,91 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Indigofera trita subsp. scabra</t>
+          <t>Hibiscus sororius</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Indigofera trita subsp. scabra</t>
+          <t>Hibiscus sororius</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Indigofera subulata var. scabra</t>
+          <t>Hibiscus sororius</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>scrambling subshrub or shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>Ha</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Iresine angustifolia</t>
+          <t>Hoffmannia nicotianifolia</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Iresine angustifolia</t>
+          <t>Hoffmannia nicotianifolia</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Iresine angustifolia</t>
+          <t>Hoffmannia nicotianifolia</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Amaranthaceae</t>
+          <t>Rubiaceae</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Iresine diffusa var. diffusa</t>
+          <t>Indigofera trita subsp. scabra</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Iresine diffusa f. diffusa</t>
+          <t>Indigofera trita subsp. scabra</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Iresine diffusa f. diffusa</t>
+          <t>Indigofera subulata var. scabra</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Amaranthaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>scrambling subshrub or shrub</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1413,22 +1413,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Kohleria tubiflora</t>
+          <t>Iresine angustifolia</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Kohleria tubiflora</t>
+          <t>Iresine angustifolia</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Kohleria tubiflora</t>
+          <t>Iresine angustifolia</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Gesneriaceae</t>
+          <t>Amaranthaceae</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1445,374 +1445,369 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Lepidaploa canescens</t>
+          <t>Iresine diffusa var. diffusa</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Lepidaploa canescens</t>
+          <t>Iresine diffusa f. diffusa</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Lepidaploa canescens</t>
+          <t>Iresine diffusa f. diffusa</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Amaranthaceae</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>scrambling shrub or liana</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Sw</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Machaerium darienense</t>
+          <t>Kohleria tubiflora</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Machaerium darienense</t>
+          <t>Kohleria tubiflora</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Machaerium darienense</t>
+          <t>Kohleria tubiflora</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Gesneriaceae</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Manettia reclinata</t>
+          <t>Lepidaploa canescens</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Manettia reclinata</t>
+          <t>Lepidaploa canescens</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Manettia reclinata</t>
+          <t>Lepidaploa canescens</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Rubiaceae</t>
+          <t>Asteraceae</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>climbing shrub</t>
+          <t>scrambling shrub or liana</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Vw</t>
+          <t>Sw</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Melochia lupulina</t>
+          <t>Machaerium darienense</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Melochia lupulina</t>
+          <t>Machaerium darienense</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Melochia lupulina</t>
+          <t>Machaerium darienense</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>L</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Melochia melissifolia</t>
+          <t>Manettia reclinata</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Melochia melissifolia</t>
+          <t>Manettia reclinata</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Melochia melissifolia</t>
+          <t>Manettia reclinata</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Rubiaceae</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>climbing shrub</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>Vw</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Mimosa casta</t>
+          <t>Melochia lupulina</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Mimosa casta</t>
+          <t>Melochia lupulina</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Mimosa casta</t>
+          <t>Melochia lupulina</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>climbing shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Vw</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Mimosa pigra</t>
+          <t>Melochia melissifolia</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Mimosa pigra</t>
+          <t>Melochia melissifolia</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Mimosa pigra</t>
+          <t>Melochia melissifolia</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Montrichardia arborescens</t>
+          <t>Mimosa casta</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Montrichardia arborescens</t>
+          <t>Mimosa casta</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Montrichardia arborescens</t>
+          <t>Mimosa casta</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Araceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>shrub or tree</t>
+          <t>climbing shrub</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Sa</t>
+          <t>Vw</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Notopleura uliginosa</t>
+          <t>Mimosa pigra</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Notopleura uliginosa</t>
+          <t>Mimosa pigra</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Notopleura uliginosa</t>
+          <t>Mimosa pigra</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Rubiaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>S</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Pavonia castaneifolia</t>
+          <t>Montrichardia arborescens</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Pavonia castaneifolia</t>
+          <t>Montrichardia arborescens</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Pavonia castaneifolia</t>
+          <t>Montrichardia arborescens</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Araceae</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>shrub or tree</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>Sa</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Pavonia paniculata</t>
+          <t>Myrcia zetekiana</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Pavonia paniculata</t>
+          <t>Myrcia zetekiana</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Pavonia paniculata</t>
+          <t>Myrcia zetekiana</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Myrtaceae</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Hw</t>
+          <t>shrub or tree</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Pavonia schiedeana</t>
+          <t>Notopleura uliginosa</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Pavonia schiedeana</t>
+          <t>Notopleura uliginosa</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Pavonia schiedeana</t>
+          <t>Notopleura uliginosa</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Rubiaceae</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1829,27 +1824,27 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Petiveria alliacea</t>
+          <t>Pavonia castaneifolia</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Petiveria alliacea</t>
+          <t>Pavonia castaneifolia</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Petiveria alliacea</t>
+          <t>Pavonia castaneifolia</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Petiveriaceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -1861,86 +1856,86 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Phoradendron quadrangulare</t>
+          <t>Pavonia paniculata</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Phoradendron quadrangulare</t>
+          <t>Pavonia paniculata</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Phoradendron quadrangulare</t>
+          <t>Pavonia paniculata</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Santalaceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>hemiparasitic shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Phytolacca rivinoides</t>
+          <t>Pavonia schiedeana</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Phytolacca rivinoides</t>
+          <t>Pavonia schiedeana</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Phytolacca rivinoides</t>
+          <t>Pavonia schiedeana</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Phytolaccaceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>perennial or shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Piper darienense</t>
+          <t>Petiveria alliacea</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Piper darienense</t>
+          <t>Petiveria alliacea</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Piper darienense</t>
+          <t>Petiveria alliacea</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Piperaceae</t>
+          <t>Petiveriaceae</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -1957,81 +1952,81 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Piper pseudogaragaranum</t>
+          <t>Phoradendron quadrangulare</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Piper pseudogaragaranum</t>
+          <t>Phoradendron quadrangulare</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Piper pseudogaragaranum</t>
+          <t>Phoradendron quadrangulare</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Piperaceae</t>
+          <t>Santalaceae</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>hemiparasitic shrub</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>PE</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Piper pubistipulum</t>
+          <t>Phytolacca rivinoides</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Piper pubistipulum</t>
+          <t>Phytolacca rivinoides</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Piper pubistipulum</t>
+          <t>Phytolacca rivinoides</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Piperaceae</t>
+          <t>Phytolaccaceae</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>perennial or shrub</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Piper trigonum</t>
+          <t>Piper darienense</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Piper trigonum</t>
+          <t>Piper darienense</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Piper trigonum</t>
+          <t>Piper darienense</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2053,17 +2048,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Piper viridicaule</t>
+          <t>Piper pseudogaragaranum</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Piper viridicaule</t>
+          <t>Piper pseudogaragaranum</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Piper viridicaule</t>
+          <t>Piper pseudogaragaranum</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2085,54 +2080,54 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Platymiscium pinnatum subsp. polystachyum</t>
+          <t>Piper pubistipulum</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Platymiscium pinnatum subsp. polystachyum</t>
+          <t>Piper pubistipulum</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Platymiscium pinnatum var. pinnatum</t>
+          <t>Piper pubistipulum</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Piperaceae</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Psychotria guapilensis</t>
+          <t>Piper trigonum</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Psychotria guapilensis</t>
+          <t>Piper trigonum</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Palicourea tonduzii</t>
+          <t>Piper trigonum</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Rubiaceae</t>
+          <t>Piperaceae</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2149,27 +2144,27 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Ronabea emetica</t>
+          <t>Piper viridicaule</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Ronabea emetica</t>
+          <t>Piper viridicaule</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Ronabea emetica</t>
+          <t>Piper viridicaule</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Rubiaceae</t>
+          <t>Piperaceae</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2181,190 +2176,286 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Schistocarpha eupatorioides</t>
+          <t>Platymiscium pinnatum subsp. polystachyum</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Schistocarpha eupatorioides</t>
+          <t>Platymiscium pinnatum subsp. polystachyum</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Schistocarpha eupatorioides</t>
+          <t>Platymiscium pinnatum var. pinnatum</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>T</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Syngonium podophyllum var. podophyllum</t>
+          <t>Psychotria guapilensis</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Syngonium podophyllum</t>
+          <t>Psychotria guapilensis</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Syngonium podophyllum</t>
+          <t>Palicourea tonduzii</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Araceae</t>
+          <t>Rubiaceae</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>liana</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Tachigali versicolor</t>
+          <t>Ronabea emetica</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Tachigali versicolor</t>
+          <t>Ronabea emetica</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Tachigali versicolor</t>
+          <t>Ronabea emetica</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Rubiaceae</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Virola multiflora</t>
+          <t>Schistocarpha eupatorioides</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Virola multiflora</t>
+          <t>Schistocarpha eupatorioides</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Virola multiflora</t>
+          <t>Schistocarpha eupatorioides</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Myristicaceae</t>
+          <t>Asteraceae</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Xanthosoma helleborifolium</t>
+          <t>Stemmadenia grandiflora</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Xanthosoma helleborifolium</t>
+          <t>Stemmadenia grandiflora</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Xanthosoma helleborifolium</t>
+          <t>Tabernaemontana grandiflora</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Araceae</t>
+          <t>Apocynaceae</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>tuberous subshrub</t>
+          <t>shrub or tree</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>U</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
+          <t>Syngonium podophyllum var. podophyllum</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Syngonium podophyllum</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Syngonium podophyllum</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Araceae</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>liana</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Tachigali versicolor</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Tachigali versicolor</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Tachigali versicolor</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Fabaceae</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>tree</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Xanthosoma helleborifolium</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Xanthosoma helleborifolium</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Xanthosoma helleborifolium</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Araceae</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>tuberous subshrub</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
           <t>Xanthosoma mexicanum</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B66" t="inlineStr">
         <is>
           <t>Xanthosoma mexicanum</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t>Xanthosoma mexicanum</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D66" t="inlineStr">
         <is>
           <t>Araceae</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t>tuberous subshrub</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F66" t="inlineStr">
         <is>
           <t>Hw</t>
         </is>

</xml_diff>

<commit_message>
fixed error with alternate names in viewtaxa like Tachigali Panamensis
</commit_message>
<xml_diff>
--- a/splists_out/needs_revision/BCI_SPECIES_POSSIBLY_WOODY_2026-03-26.xlsx
+++ b/splists_out/needs_revision/BCI_SPECIES_POSSIBLY_WOODY_2026-03-26.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -773,81 +773,81 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cestrum megalophyllum</t>
+          <t>Chamissoa altissima</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cestrum megalophyllum</t>
+          <t>Chamissoa altissima</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Cestrum megalophyllum</t>
+          <t>Chamissoa altissima</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Solanaceae</t>
+          <t>Amaranthaceae</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>shrub or tree</t>
+          <t>scrambling subshrub or shrub</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Chamissoa altissima</t>
+          <t>Clibadium surinamense</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Chamissoa altissima</t>
+          <t>Clibadium surinamense</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Chamissoa altissima</t>
+          <t>Clibadium surinamense</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Amaranthaceae</t>
+          <t>Asteraceae</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>scrambling subshrub or shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>Sw</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Clibadium surinamense</t>
+          <t>Clibadium sylvestre</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Clibadium surinamense</t>
+          <t>Clibadium sylvestre</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Clibadium surinamense</t>
+          <t>Clibadium sylvestre</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>scrambling shrub or tree</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -869,113 +869,113 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Clibadium sylvestre</t>
+          <t>Corchorus siliquosus</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Clibadium sylvestre</t>
+          <t>Corchorus siliquosus</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Clibadium sylvestre</t>
+          <t>Corchorus siliquosus</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>scrambling shrub or tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Sw</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Corchorus siliquosus</t>
+          <t>Coussapoa asperifolia subsp. magnifolia</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Corchorus siliquosus</t>
+          <t>Coussapoa asperifolia subsp. magnifolia</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Corchorus siliquosus</t>
+          <t>Coussapoa asperifolia subsp. magnifolia</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Urticaceae</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>E</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Coussapoa asperifolia subsp. magnifolia</t>
+          <t>Crotalaria cajanifolia</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Coussapoa asperifolia subsp. magnifolia</t>
+          <t>Crotalaria cajanifolia</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Coussapoa asperifolia subsp. magnifolia</t>
+          <t>Crotalaria cajanifolia</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Urticaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Crotalaria cajanifolia</t>
+          <t>Dalbergia brownei</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Crotalaria cajanifolia</t>
+          <t>Dalbergia brownei</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Crotalaria cajanifolia</t>
+          <t>Dalbergia brownei</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -985,34 +985,34 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>shrub or tree</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>L</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Dalbergia brownei</t>
+          <t>Dendropanax stenodontus</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Dalbergia brownei</t>
+          <t>Dendropanax stenodontus</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Dalbergia brownei</t>
+          <t>Dendropanax stenodontus</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Araliaceae</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1022,56 +1022,56 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Dendropanax stenodontus</t>
+          <t>Desmodium cajanifolium</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dendropanax stenodontus</t>
+          <t>Desmodium cajanifolium</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Dendropanax stenodontus</t>
+          <t>Desmodium cajanifolium</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Araliaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>shrub or tree</t>
+          <t>perennial or shrub</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Sw</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Desmodium cajanifolium</t>
+          <t>Desmodium distortum</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Desmodium cajanifolium</t>
+          <t>Desmodium distortum</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Desmodium cajanifolium</t>
+          <t>Desmodium distortum</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1081,29 +1081,29 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>perennial or shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Sw</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Desmodium distortum</t>
+          <t>Desmodium wydlerianum</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Desmodium distortum</t>
+          <t>Desmodium wydlerianum</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Desmodium distortum</t>
+          <t>Desmodium wydlerianum</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1113,39 +1113,39 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Desmodium wydlerianum</t>
+          <t>Dieffenbachia longispatha</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Desmodium wydlerianum</t>
+          <t>Dieffenbachia longispatha</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Desmodium wydlerianum</t>
+          <t>Dieffenbachia longispatha</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Araceae</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1157,155 +1157,155 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Dieffenbachia longispatha</t>
+          <t>Ficus dugandii</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Dieffenbachia longispatha</t>
+          <t>Ficus dugandii</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Dieffenbachia longispatha</t>
+          <t>Ficus dugandii</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Araceae</t>
+          <t>Moraceae</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>TE</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Ficus bullenei</t>
+          <t>Hebeclinium macrophyllum</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Ficus bullenei</t>
+          <t>Hebeclinium macrophyllum</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Ficus bullenei</t>
+          <t>Hebeclinium macrophyllum</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Moraceae</t>
+          <t>Asteraceae</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ficus dugandii</t>
+          <t>Herpetacanthus panamensis</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Ficus dugandii</t>
+          <t>Herpetacanthus panamensis</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Ficus dugandii</t>
+          <t>Herpetacanthus panamensis</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Moraceae</t>
+          <t>Acanthaceae</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Hebeclinium macrophyllum</t>
+          <t>Hibiscus sororius</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Hebeclinium macrophyllum</t>
+          <t>Hibiscus sororius</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Hebeclinium macrophyllum</t>
+          <t>Hibiscus sororius</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>Ha</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Herpetacanthus panamensis</t>
+          <t>Hoffmannia nicotianifolia</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Herpetacanthus panamensis</t>
+          <t>Hoffmannia nicotianifolia</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Herpetacanthus panamensis</t>
+          <t>Hoffmannia nicotianifolia</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Acanthaceae</t>
+          <t>Rubiaceae</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1317,91 +1317,91 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Hibiscus sororius</t>
+          <t>Indigofera trita subsp. scabra</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Hibiscus sororius</t>
+          <t>Indigofera trita subsp. scabra</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Hibiscus sororius</t>
+          <t>Indigofera subulata var. scabra</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>scrambling subshrub or shrub</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Ha</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Hoffmannia nicotianifolia</t>
+          <t>Iresine angustifolia</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Hoffmannia nicotianifolia</t>
+          <t>Iresine angustifolia</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Hoffmannia nicotianifolia</t>
+          <t>Iresine angustifolia</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Rubiaceae</t>
+          <t>Amaranthaceae</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Indigofera trita subsp. scabra</t>
+          <t>Iresine diffusa var. diffusa</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Indigofera trita subsp. scabra</t>
+          <t>Iresine diffusa f. diffusa</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Indigofera subulata var. scabra</t>
+          <t>Iresine diffusa f. diffusa</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Amaranthaceae</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>scrambling subshrub or shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1413,22 +1413,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Iresine angustifolia</t>
+          <t>Kohleria tubiflora</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Iresine angustifolia</t>
+          <t>Kohleria tubiflora</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Iresine angustifolia</t>
+          <t>Kohleria tubiflora</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Amaranthaceae</t>
+          <t>Gesneriaceae</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1445,369 +1445,374 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Iresine diffusa var. diffusa</t>
+          <t>Lepidaploa canescens</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Iresine diffusa f. diffusa</t>
+          <t>Lepidaploa canescens</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Iresine diffusa f. diffusa</t>
+          <t>Lepidaploa canescens</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Amaranthaceae</t>
+          <t>Asteraceae</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>scrambling shrub or liana</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>Sw</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Kohleria tubiflora</t>
+          <t>Machaerium darienense</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Kohleria tubiflora</t>
+          <t>Machaerium darienense</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Kohleria tubiflora</t>
+          <t>Machaerium darienense</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Gesneriaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>L</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Lepidaploa canescens</t>
+          <t>Manettia reclinata</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Lepidaploa canescens</t>
+          <t>Manettia reclinata</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Lepidaploa canescens</t>
+          <t>Manettia reclinata</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Rubiaceae</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>scrambling shrub or liana</t>
+          <t>climbing shrub</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Sw</t>
+          <t>Vw</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Machaerium darienense</t>
+          <t>Melochia lupulina</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Machaerium darienense</t>
+          <t>Melochia lupulina</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Machaerium darienense</t>
+          <t>Melochia lupulina</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Manettia reclinata</t>
+          <t>Melochia melissifolia</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Manettia reclinata</t>
+          <t>Melochia melissifolia</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Manettia reclinata</t>
+          <t>Melochia melissifolia</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Rubiaceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>climbing shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Vw</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Melochia lupulina</t>
+          <t>Mimosa casta</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Melochia lupulina</t>
+          <t>Mimosa casta</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Melochia lupulina</t>
+          <t>Mimosa casta</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>climbing shrub</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>Vw</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Melochia melissifolia</t>
+          <t>Mimosa pigra</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Melochia melissifolia</t>
+          <t>Mimosa pigra</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Melochia melissifolia</t>
+          <t>Mimosa pigra</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>S</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mimosa casta</t>
+          <t>Montrichardia arborescens</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Mimosa casta</t>
+          <t>Montrichardia arborescens</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Mimosa casta</t>
+          <t>Montrichardia arborescens</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Araceae</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>climbing shrub</t>
+          <t>shrub or tree</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Vw</t>
+          <t>Sa</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mimosa pigra</t>
+          <t>Notopleura uliginosa</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Mimosa pigra</t>
+          <t>Notopleura uliginosa</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mimosa pigra</t>
+          <t>Notopleura uliginosa</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Rubiaceae</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Montrichardia arborescens</t>
+          <t>Pavonia castaneifolia</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Montrichardia arborescens</t>
+          <t>Pavonia castaneifolia</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Montrichardia arborescens</t>
+          <t>Pavonia castaneifolia</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Araceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>shrub or tree</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Sa</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Myrcia zetekiana</t>
+          <t>Pavonia paniculata</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Myrcia zetekiana</t>
+          <t>Pavonia paniculata</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Myrcia zetekiana</t>
+          <t>Pavonia paniculata</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Myrtaceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>shrub or tree</t>
+          <t>subshrub or shrub</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Notopleura uliginosa</t>
+          <t>Pavonia schiedeana</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Notopleura uliginosa</t>
+          <t>Pavonia schiedeana</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Notopleura uliginosa</t>
+          <t>Pavonia schiedeana</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Rubiaceae</t>
+          <t>Malvaceae</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1824,27 +1829,27 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Pavonia castaneifolia</t>
+          <t>Petiveria alliacea</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Pavonia castaneifolia</t>
+          <t>Petiveria alliacea</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Pavonia castaneifolia</t>
+          <t>Petiveria alliacea</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Petiveriaceae</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -1856,86 +1861,86 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Pavonia paniculata</t>
+          <t>Phoradendron quadrangulare</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Pavonia paniculata</t>
+          <t>Phoradendron quadrangulare</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Pavonia paniculata</t>
+          <t>Phoradendron quadrangulare</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Santalaceae</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>hemiparasitic shrub</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>PE</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Pavonia schiedeana</t>
+          <t>Phytolacca rivinoides</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Pavonia schiedeana</t>
+          <t>Phytolacca rivinoides</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Pavonia schiedeana</t>
+          <t>Phytolacca rivinoides</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Malvaceae</t>
+          <t>Phytolaccaceae</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>perennial or shrub</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Petiveria alliacea</t>
+          <t>Piper darienense</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Petiveria alliacea</t>
+          <t>Piper darienense</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Petiveria alliacea</t>
+          <t>Piper darienense</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Petiveriaceae</t>
+          <t>Piperaceae</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -1952,81 +1957,81 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Phoradendron quadrangulare</t>
+          <t>Piper pseudogaragaranum</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Phoradendron quadrangulare</t>
+          <t>Piper pseudogaragaranum</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Phoradendron quadrangulare</t>
+          <t>Piper pseudogaragaranum</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Santalaceae</t>
+          <t>Piperaceae</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>hemiparasitic shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Phytolacca rivinoides</t>
+          <t>Piper pubistipulum</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Phytolacca rivinoides</t>
+          <t>Piper pubistipulum</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Phytolacca rivinoides</t>
+          <t>Piper pubistipulum</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Phytolaccaceae</t>
+          <t>Piperaceae</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>perennial or shrub</t>
+          <t>shrub</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Piper darienense</t>
+          <t>Piper trigonum</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Piper darienense</t>
+          <t>Piper trigonum</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Piper darienense</t>
+          <t>Piper trigonum</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2048,17 +2053,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Piper pseudogaragaranum</t>
+          <t>Piper viridicaule</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Piper pseudogaragaranum</t>
+          <t>Piper viridicaule</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Piper pseudogaragaranum</t>
+          <t>Piper viridicaule</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2080,54 +2085,54 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Piper pubistipulum</t>
+          <t>Platymiscium pinnatum subsp. polystachyum</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Piper pubistipulum</t>
+          <t>Platymiscium pinnatum subsp. polystachyum</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Piper pubistipulum</t>
+          <t>Platymiscium pinnatum var. pinnatum</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Piperaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>T</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Piper trigonum</t>
+          <t>Psychotria guapilensis</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Piper trigonum</t>
+          <t>Psychotria guapilensis</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Piper trigonum</t>
+          <t>Palicourea tonduzii</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Piperaceae</t>
+          <t>Rubiaceae</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2144,27 +2149,27 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Piper viridicaule</t>
+          <t>Ronabea emetica</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Piper viridicaule</t>
+          <t>Ronabea emetica</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Piper viridicaule</t>
+          <t>Ronabea emetica</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Piperaceae</t>
+          <t>Rubiaceae</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>shrub</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2176,286 +2181,158 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Platymiscium pinnatum subsp. polystachyum</t>
+          <t>Schistocarpha eupatorioides</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Platymiscium pinnatum subsp. polystachyum</t>
+          <t>Schistocarpha eupatorioides</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Platymiscium pinnatum var. pinnatum</t>
+          <t>Schistocarpha eupatorioides</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Asteraceae</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>Hw</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Psychotria guapilensis</t>
+          <t>Syngonium podophyllum var. podophyllum</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Psychotria guapilensis</t>
+          <t>Syngonium podophyllum</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Palicourea tonduzii</t>
+          <t>Syngonium podophyllum</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Rubiaceae</t>
+          <t>Araceae</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>liana</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>E</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Ronabea emetica</t>
+          <t>Tachigali versicolor</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Ronabea emetica</t>
+          <t>Tachigali versicolor</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Ronabea emetica</t>
+          <t>Tachigali versicolor</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Rubiaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>tree</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>T</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Schistocarpha eupatorioides</t>
+          <t>Xanthosoma helleborifolium</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Schistocarpha eupatorioides</t>
+          <t>Xanthosoma helleborifolium</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Schistocarpha eupatorioides</t>
+          <t>Xanthosoma helleborifolium</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Araceae</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>tuberous subshrub</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>H</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Stemmadenia grandiflora</t>
+          <t>Xanthosoma mexicanum</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Stemmadenia grandiflora</t>
+          <t>Xanthosoma mexicanum</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Tabernaemontana grandiflora</t>
+          <t>Xanthosoma mexicanum</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Apocynaceae</t>
+          <t>Araceae</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>shrub or tree</t>
+          <t>tuberous subshrub</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Syngonium podophyllum var. podophyllum</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Syngonium podophyllum</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Syngonium podophyllum</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Araceae</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>liana</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Tachigali versicolor</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Tachigali versicolor</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Tachigali versicolor</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Fabaceae</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>tree</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Xanthosoma helleborifolium</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Xanthosoma helleborifolium</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Xanthosoma helleborifolium</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Araceae</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>tuberous subshrub</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Xanthosoma mexicanum</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Xanthosoma mexicanum</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Xanthosoma mexicanum</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Araceae</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>tuberous subshrub</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
         <is>
           <t>Hw</t>
         </is>

</xml_diff>